<commit_message>
Adding Payback Excel file
</commit_message>
<xml_diff>
--- a/Excel FIles/Assignment1_Excel.xlsx
+++ b/Excel FIles/Assignment1_Excel.xlsx
@@ -5,19 +5,21 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MVIC\(BIT 301)_IT Project Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MVIC\(BIT 301)_IT Project Management\Excel FIles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4A9A80-B559-4921-A3B9-0FD727D07A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCCD207-F795-4360-9375-B3C4C9F18079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{151C8DFF-D34E-46B5-935E-790C9F0A2CD3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{151C8DFF-D34E-46B5-935E-790C9F0A2CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Financial Analysis" sheetId="1" r:id="rId1"/>
     <sheet name="Cost Estimate" sheetId="2" r:id="rId2"/>
+    <sheet name="Payback" sheetId="3" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="108">
   <si>
     <t>Financial Analysis for EcoPantry: Smart Inventory and Food Sharing application to Reduce Food Waste</t>
   </si>
@@ -345,6 +347,30 @@
   </si>
   <si>
     <t>Weekly Cost Breakdown</t>
+  </si>
+  <si>
+    <t>Note: Discounted costs and benefits below are taken from the Financial Analysis (Business Case).</t>
+  </si>
+  <si>
+    <t>Years 0-3 = project development year plus three post-launch years. Discount rate: 8%.</t>
+  </si>
+  <si>
+    <t>Costs</t>
+  </si>
+  <si>
+    <t>Benefits</t>
+  </si>
+  <si>
+    <t>Cum Costs</t>
+  </si>
+  <si>
+    <t>Cum Benefits</t>
+  </si>
+  <si>
+    <t>Created by: EcoPantry Team</t>
+  </si>
+  <si>
+    <t>Payback Period Chart for EcoPantry</t>
   </si>
 </sst>
 </file>
@@ -360,7 +386,7 @@
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,6 +507,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -658,7 +692,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -713,57 +747,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -790,17 +779,79 @@
     </xf>
     <xf numFmtId="164" fontId="15" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="8" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="166" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -811,6 +862,1031 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Payback – EcoPantry</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Payback!$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Year</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Payback!$A$7:$A$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3323-4BBF-8D93-391013B4079C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Payback!$D$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Cum Costs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Payback!$D$7:$D$10</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>18480</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>25887</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>33432</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>41116</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3323-4BBF-8D93-391013B4079C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Payback!$E$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Cum Benefits</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Payback!$E$7:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>32407</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>80418</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>147100</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-3323-4BBF-8D93-391013B4079C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1219650351"/>
+        <c:axId val="1234010959"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1219650351"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1234010959"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1234010959"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1219650351"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -987,6 +2063,47 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>682625</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>746125</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>30163</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBF7A65A-71A6-68E4-216F-A9D86300E846}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -1009,6 +2126,85 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+      <sheetName val="Sheet2"/>
+      <sheetName val="Sheet3"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="7">
+          <cell r="A7">
+            <v>0</v>
+          </cell>
+          <cell r="D7">
+            <v>18480</v>
+          </cell>
+          <cell r="E7">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="A8">
+            <v>1</v>
+          </cell>
+          <cell r="D8">
+            <v>25887.407407407409</v>
+          </cell>
+          <cell r="E8">
+            <v>32407.407407407401</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="A9">
+            <v>2</v>
+          </cell>
+          <cell r="D9">
+            <v>33431.9890260631</v>
+          </cell>
+          <cell r="E9">
+            <v>80418.381344307301</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="A10">
+            <v>3</v>
+          </cell>
+          <cell r="D10">
+            <v>41116.285119138338</v>
+          </cell>
+          <cell r="E10">
+            <v>147100.28959000151</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC6639B1-3DD7-41B5-8ADE-B29CB10F8394}" name="Table1" displayName="Table1" ref="A6:E10" totalsRowShown="0">
+  <autoFilter ref="A6:E10" xr:uid="{FC6639B1-3DD7-41B5-8ADE-B29CB10F8394}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{9B77C32C-F3D8-443E-B0D0-0CD47E8ADF4F}" name="Year"/>
+    <tableColumn id="2" xr3:uid="{65EE8341-11D6-43B2-9F5E-10560FABE0F0}" name="Costs" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{2F5E6A88-02C6-4AB9-B314-B4CD1E127DEA}" name="Benefits" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{95DE8CD5-69A7-436D-AE76-53ECF29EDD31}" name="Cum Costs" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{020C4A80-1499-4E26-847F-1AD4554936DB}" name="Cum Benefits" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1341,15 +2537,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="22.8">
-      <c r="A1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
+      <c r="A1" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
     </row>
     <row r="2" spans="1:7" ht="22.8">
       <c r="A2" s="1" t="s">
@@ -1367,13 +2563,13 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" ht="15.6">
-      <c r="A3" s="44"/>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
+      <c r="A3" s="72"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3"/>
@@ -1400,12 +2596,12 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="7"/>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
       <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:7">
@@ -1486,7 +2682,7 @@
         <f>E9*E10</f>
         <v>7684.2960930752415</v>
       </c>
-      <c r="F11" s="78">
+      <c r="F11" s="62">
         <f>SUM(B11:E11)</f>
         <v>41116.285119138338</v>
       </c>
@@ -1559,7 +2755,7 @@
         <f>E13*E14</f>
         <v>66681.908245694241</v>
       </c>
-      <c r="F15" s="78">
+      <c r="F15" s="62">
         <f>SUM(B15:E15)</f>
         <v>147100.28959000151</v>
       </c>
@@ -1592,7 +2788,7 @@
         <f>E15-E11</f>
         <v>58997.612152618996</v>
       </c>
-      <c r="F17" s="76">
+      <c r="F17" s="61">
         <f>SUM(B17:E17)</f>
         <v>105984.00447086316</v>
       </c>
@@ -1632,23 +2828,23 @@
       <c r="A20" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="77">
+      <c r="B20" s="75">
         <f>F17/F11</f>
         <v>2.577664887860478</v>
       </c>
-      <c r="C20" s="77"/>
-      <c r="D20" s="77"/>
-      <c r="E20" s="77"/>
-      <c r="F20" s="77"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="75"/>
+      <c r="E20" s="75"/>
+      <c r="F20" s="75"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="B21" s="47" t="s">
+      <c r="B21" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="47"/>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="47"/>
+      <c r="C21" s="76"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
@@ -1656,70 +2852,70 @@
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="42" t="s">
+      <c r="A25" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
+      <c r="B25" s="65"/>
+      <c r="C25" s="65"/>
+      <c r="D25" s="65"/>
+      <c r="E25" s="65"/>
+      <c r="F25" s="65"/>
+      <c r="G25" s="65"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="42" t="s">
+      <c r="A26" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="42"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
-      <c r="G26" s="42"/>
+      <c r="B26" s="65"/>
+      <c r="C26" s="65"/>
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="65"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="42" t="s">
+      <c r="A27" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="42"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="42"/>
-      <c r="F27" s="42"/>
-      <c r="G27" s="42"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="65"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="65"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
+      <c r="B28" s="65"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="65"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="42" t="s">
+      <c r="A29" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42"/>
+      <c r="B29" s="65"/>
+      <c r="C29" s="65"/>
+      <c r="D29" s="65"/>
+      <c r="E29" s="65"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
+      <c r="B30" s="65"/>
+      <c r="C30" s="65"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="65"/>
+      <c r="F30" s="65"/>
+      <c r="G30" s="65"/>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="38" t="s">
@@ -1747,24 +2943,24 @@
       </c>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" s="40" t="s">
+      <c r="A39" s="77" t="s">
         <v>63</v>
       </c>
-      <c r="B39" s="41"/>
-      <c r="C39" s="41"/>
+      <c r="B39" s="78"/>
+      <c r="C39" s="78"/>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" s="41"/>
-      <c r="B40" s="41"/>
-      <c r="C40" s="41"/>
+      <c r="A40" s="78"/>
+      <c r="B40" s="78"/>
+      <c r="C40" s="78"/>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="40" t="s">
+      <c r="A41" s="77" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="41"/>
+      <c r="A42" s="78"/>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
@@ -1786,12 +2982,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B21:F21"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A27:G27"/>
@@ -1799,6 +2989,12 @@
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A39:C40"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B21:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1823,18 +3019,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="21">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
     </row>
     <row r="2" spans="1:30" ht="36" customHeight="1">
       <c r="A2" s="25" t="s">
@@ -1870,25 +3066,25 @@
       <c r="H5" s="22"/>
       <c r="I5" s="22"/>
       <c r="J5" s="22"/>
-      <c r="N5" s="58" t="s">
+      <c r="N5" s="63" t="s">
         <v>99</v>
       </c>
-      <c r="O5" s="57"/>
-      <c r="P5" s="57"/>
-      <c r="Q5" s="57"/>
-      <c r="R5" s="57"/>
-      <c r="S5" s="57"/>
-      <c r="T5" s="57"/>
-      <c r="U5" s="57"/>
-      <c r="V5" s="57"/>
-      <c r="W5" s="57"/>
-      <c r="X5" s="57"/>
-      <c r="Y5" s="57"/>
-      <c r="Z5" s="57"/>
-      <c r="AA5" s="57"/>
-      <c r="AB5" s="57"/>
-      <c r="AC5" s="57"/>
-      <c r="AD5" s="57"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+      <c r="Q5" s="64"/>
+      <c r="R5" s="64"/>
+      <c r="S5" s="64"/>
+      <c r="T5" s="64"/>
+      <c r="U5" s="64"/>
+      <c r="V5" s="64"/>
+      <c r="W5" s="64"/>
+      <c r="X5" s="64"/>
+      <c r="Y5" s="64"/>
+      <c r="Z5" s="64"/>
+      <c r="AA5" s="64"/>
+      <c r="AB5" s="64"/>
+      <c r="AC5" s="64"/>
+      <c r="AD5" s="64"/>
     </row>
     <row r="6" spans="1:30">
       <c r="B6" s="22"/>
@@ -1903,82 +3099,82 @@
     </row>
     <row r="7" spans="1:30">
       <c r="A7" s="37"/>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="51" t="s">
+      <c r="C7" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="51" t="s">
+      <c r="D7" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="51" t="s">
+      <c r="F7" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="49" t="s">
+      <c r="G7" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="49" t="s">
+      <c r="H7" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="51" t="s">
+      <c r="I7" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="J7" s="51" t="s">
+      <c r="J7" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="N7" s="62" t="s">
+      <c r="N7" s="47" t="s">
         <v>68</v>
       </c>
-      <c r="O7" s="63" t="s">
+      <c r="O7" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="P7" s="63" t="s">
+      <c r="P7" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="Q7" s="63" t="s">
+      <c r="Q7" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="R7" s="63" t="s">
+      <c r="R7" s="48" t="s">
         <v>72</v>
       </c>
-      <c r="S7" s="63" t="s">
+      <c r="S7" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="T7" s="63" t="s">
+      <c r="T7" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="U7" s="63" t="s">
+      <c r="U7" s="48" t="s">
         <v>75</v>
       </c>
-      <c r="V7" s="63" t="s">
+      <c r="V7" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="W7" s="63" t="s">
+      <c r="W7" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="X7" s="63" t="s">
+      <c r="X7" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="Y7" s="63" t="s">
+      <c r="Y7" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="Z7" s="63" t="s">
+      <c r="Z7" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="AA7" s="63" t="s">
+      <c r="AA7" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="AB7" s="63" t="s">
+      <c r="AB7" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="AC7" s="64" t="s">
+      <c r="AC7" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="AD7" s="64" t="s">
+      <c r="AD7" s="49" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1986,41 +3182,41 @@
       <c r="A8" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="50"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
+      <c r="B8" s="68"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="68"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="70"/>
       <c r="N8" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="O8" s="59">
+      <c r="O8" s="44">
         <v>25</v>
       </c>
-      <c r="P8" s="59">
+      <c r="P8" s="44">
         <v>15</v>
       </c>
-      <c r="Q8" s="59"/>
-      <c r="R8" s="59"/>
-      <c r="S8" s="59"/>
-      <c r="T8" s="59"/>
-      <c r="U8" s="59"/>
-      <c r="V8" s="59"/>
-      <c r="W8" s="59"/>
-      <c r="X8" s="59"/>
-      <c r="Y8" s="59"/>
-      <c r="Z8" s="59"/>
-      <c r="AA8" s="59"/>
-      <c r="AB8" s="59"/>
-      <c r="AC8" s="60">
+      <c r="Q8" s="44"/>
+      <c r="R8" s="44"/>
+      <c r="S8" s="44"/>
+      <c r="T8" s="44"/>
+      <c r="U8" s="44"/>
+      <c r="V8" s="44"/>
+      <c r="W8" s="44"/>
+      <c r="X8" s="44"/>
+      <c r="Y8" s="44"/>
+      <c r="Z8" s="44"/>
+      <c r="AA8" s="44"/>
+      <c r="AB8" s="44"/>
+      <c r="AC8" s="45">
         <f t="shared" ref="AC8:AC19" si="0">SUM(O8:AB8)</f>
         <v>40</v>
       </c>
-      <c r="AD8" s="61">
+      <c r="AD8" s="46">
         <f>AC8*'[1]Cost Estimate Summary'!$B$5</f>
         <v>800</v>
       </c>
@@ -2064,31 +3260,31 @@
       <c r="N9" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="O9" s="53"/>
-      <c r="P9" s="53">
+      <c r="O9" s="40"/>
+      <c r="P9" s="40">
         <v>15</v>
       </c>
-      <c r="Q9" s="53">
+      <c r="Q9" s="40">
         <v>45</v>
       </c>
-      <c r="R9" s="53">
+      <c r="R9" s="40">
         <v>30</v>
       </c>
-      <c r="S9" s="53"/>
-      <c r="T9" s="53"/>
-      <c r="U9" s="53"/>
-      <c r="V9" s="53"/>
-      <c r="W9" s="53"/>
-      <c r="X9" s="53"/>
-      <c r="Y9" s="53"/>
-      <c r="Z9" s="53"/>
-      <c r="AA9" s="53"/>
-      <c r="AB9" s="53"/>
-      <c r="AC9" s="54">
+      <c r="S9" s="40"/>
+      <c r="T9" s="40"/>
+      <c r="U9" s="40"/>
+      <c r="V9" s="40"/>
+      <c r="W9" s="40"/>
+      <c r="X9" s="40"/>
+      <c r="Y9" s="40"/>
+      <c r="Z9" s="40"/>
+      <c r="AA9" s="40"/>
+      <c r="AB9" s="40"/>
+      <c r="AC9" s="41">
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="AD9" s="55">
+      <c r="AD9" s="42">
         <f>AC9*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1800</v>
       </c>
@@ -2132,29 +3328,29 @@
       <c r="N10" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="O10" s="53"/>
-      <c r="P10" s="53"/>
-      <c r="Q10" s="53"/>
-      <c r="R10" s="53">
+      <c r="O10" s="40"/>
+      <c r="P10" s="40"/>
+      <c r="Q10" s="40"/>
+      <c r="R10" s="40">
         <v>10</v>
       </c>
-      <c r="S10" s="53">
+      <c r="S10" s="40">
         <v>30</v>
       </c>
-      <c r="T10" s="53"/>
-      <c r="U10" s="53"/>
-      <c r="V10" s="53"/>
-      <c r="W10" s="53"/>
-      <c r="X10" s="53"/>
-      <c r="Y10" s="53"/>
-      <c r="Z10" s="53"/>
-      <c r="AA10" s="53"/>
-      <c r="AB10" s="53"/>
-      <c r="AC10" s="54">
+      <c r="T10" s="40"/>
+      <c r="U10" s="40"/>
+      <c r="V10" s="40"/>
+      <c r="W10" s="40"/>
+      <c r="X10" s="40"/>
+      <c r="Y10" s="40"/>
+      <c r="Z10" s="40"/>
+      <c r="AA10" s="40"/>
+      <c r="AB10" s="40"/>
+      <c r="AC10" s="41">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="AD10" s="55">
+      <c r="AD10" s="42">
         <f>AC10*'[1]Cost Estimate Summary'!$B$5</f>
         <v>800</v>
       </c>
@@ -2175,29 +3371,29 @@
       <c r="N11" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="O11" s="53"/>
-      <c r="P11" s="53"/>
-      <c r="Q11" s="53"/>
-      <c r="R11" s="53"/>
-      <c r="S11" s="53">
+      <c r="O11" s="40"/>
+      <c r="P11" s="40"/>
+      <c r="Q11" s="40"/>
+      <c r="R11" s="40"/>
+      <c r="S11" s="40">
         <v>20</v>
       </c>
-      <c r="T11" s="53">
+      <c r="T11" s="40">
         <v>30</v>
       </c>
-      <c r="U11" s="53"/>
-      <c r="V11" s="53"/>
-      <c r="W11" s="53"/>
-      <c r="X11" s="53"/>
-      <c r="Y11" s="53"/>
-      <c r="Z11" s="53"/>
-      <c r="AA11" s="53"/>
-      <c r="AB11" s="53"/>
-      <c r="AC11" s="54">
+      <c r="U11" s="40"/>
+      <c r="V11" s="40"/>
+      <c r="W11" s="40"/>
+      <c r="X11" s="40"/>
+      <c r="Y11" s="40"/>
+      <c r="Z11" s="40"/>
+      <c r="AA11" s="40"/>
+      <c r="AB11" s="40"/>
+      <c r="AC11" s="41">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="AD11" s="55">
+      <c r="AD11" s="42">
         <f>AC11*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1000</v>
       </c>
@@ -2241,29 +3437,29 @@
       <c r="N12" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="O12" s="53"/>
-      <c r="P12" s="53"/>
-      <c r="Q12" s="53"/>
-      <c r="R12" s="53"/>
-      <c r="S12" s="53"/>
-      <c r="T12" s="53">
+      <c r="O12" s="40"/>
+      <c r="P12" s="40"/>
+      <c r="Q12" s="40"/>
+      <c r="R12" s="40"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="40">
         <v>15</v>
       </c>
-      <c r="U12" s="53">
+      <c r="U12" s="40">
         <v>25</v>
       </c>
-      <c r="V12" s="53"/>
-      <c r="W12" s="53"/>
-      <c r="X12" s="53"/>
-      <c r="Y12" s="53"/>
-      <c r="Z12" s="53"/>
-      <c r="AA12" s="53"/>
-      <c r="AB12" s="53"/>
-      <c r="AC12" s="54">
+      <c r="V12" s="40"/>
+      <c r="W12" s="40"/>
+      <c r="X12" s="40"/>
+      <c r="Y12" s="40"/>
+      <c r="Z12" s="40"/>
+      <c r="AA12" s="40"/>
+      <c r="AB12" s="40"/>
+      <c r="AC12" s="41">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="AD12" s="55">
+      <c r="AD12" s="42">
         <f>AC12*'[1]Cost Estimate Summary'!$B$5</f>
         <v>800</v>
       </c>
@@ -2307,33 +3503,33 @@
       <c r="N13" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="O13" s="53"/>
-      <c r="P13" s="53"/>
-      <c r="Q13" s="53"/>
-      <c r="R13" s="53"/>
-      <c r="S13" s="53"/>
-      <c r="T13" s="53">
+      <c r="O13" s="40"/>
+      <c r="P13" s="40"/>
+      <c r="Q13" s="40"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="40">
         <v>10</v>
       </c>
-      <c r="U13" s="53">
+      <c r="U13" s="40">
         <v>25</v>
       </c>
-      <c r="V13" s="53">
+      <c r="V13" s="40">
         <v>40</v>
       </c>
-      <c r="W13" s="53">
+      <c r="W13" s="40">
         <v>45</v>
       </c>
-      <c r="X13" s="53"/>
-      <c r="Y13" s="53"/>
-      <c r="Z13" s="53"/>
-      <c r="AA13" s="53"/>
-      <c r="AB13" s="53"/>
-      <c r="AC13" s="54">
+      <c r="X13" s="40"/>
+      <c r="Y13" s="40"/>
+      <c r="Z13" s="40"/>
+      <c r="AA13" s="40"/>
+      <c r="AB13" s="40"/>
+      <c r="AC13" s="41">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="AD13" s="55">
+      <c r="AD13" s="42">
         <f>AC13*'[1]Cost Estimate Summary'!$B$5</f>
         <v>2400</v>
       </c>
@@ -2377,33 +3573,33 @@
       <c r="N14" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="O14" s="53"/>
-      <c r="P14" s="53"/>
-      <c r="Q14" s="53"/>
-      <c r="R14" s="53"/>
-      <c r="S14" s="53"/>
-      <c r="T14" s="53">
+      <c r="O14" s="40"/>
+      <c r="P14" s="40"/>
+      <c r="Q14" s="40"/>
+      <c r="R14" s="40"/>
+      <c r="S14" s="40"/>
+      <c r="T14" s="40">
         <v>15</v>
       </c>
-      <c r="U14" s="53">
+      <c r="U14" s="40">
         <v>30</v>
       </c>
-      <c r="V14" s="53">
+      <c r="V14" s="40">
         <v>45</v>
       </c>
-      <c r="W14" s="53">
+      <c r="W14" s="40">
         <v>40</v>
       </c>
-      <c r="X14" s="53"/>
-      <c r="Y14" s="53"/>
-      <c r="Z14" s="53"/>
-      <c r="AA14" s="53"/>
-      <c r="AB14" s="53"/>
-      <c r="AC14" s="54">
+      <c r="X14" s="40"/>
+      <c r="Y14" s="40"/>
+      <c r="Z14" s="40"/>
+      <c r="AA14" s="40"/>
+      <c r="AB14" s="40"/>
+      <c r="AC14" s="41">
         <f t="shared" si="0"/>
         <v>130</v>
       </c>
-      <c r="AD14" s="55">
+      <c r="AD14" s="42">
         <f>AC14*'[1]Cost Estimate Summary'!$B$5</f>
         <v>2600</v>
       </c>
@@ -2447,29 +3643,29 @@
       <c r="N15" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="O15" s="53"/>
-      <c r="P15" s="53"/>
-      <c r="Q15" s="53"/>
-      <c r="R15" s="53"/>
-      <c r="S15" s="53"/>
-      <c r="T15" s="53"/>
-      <c r="U15" s="53"/>
-      <c r="V15" s="53"/>
-      <c r="W15" s="53">
+      <c r="O15" s="40"/>
+      <c r="P15" s="40"/>
+      <c r="Q15" s="40"/>
+      <c r="R15" s="40"/>
+      <c r="S15" s="40"/>
+      <c r="T15" s="40"/>
+      <c r="U15" s="40"/>
+      <c r="V15" s="40"/>
+      <c r="W15" s="40">
         <v>15</v>
       </c>
-      <c r="X15" s="53">
+      <c r="X15" s="40">
         <v>25</v>
       </c>
-      <c r="Y15" s="53"/>
-      <c r="Z15" s="53"/>
-      <c r="AA15" s="53"/>
-      <c r="AB15" s="53"/>
-      <c r="AC15" s="54">
+      <c r="Y15" s="40"/>
+      <c r="Z15" s="40"/>
+      <c r="AA15" s="40"/>
+      <c r="AB15" s="40"/>
+      <c r="AC15" s="41">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="AD15" s="55">
+      <c r="AD15" s="42">
         <f>AC15*'[1]Cost Estimate Summary'!$B$5</f>
         <v>800</v>
       </c>
@@ -2513,29 +3709,29 @@
       <c r="N16" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="O16" s="53"/>
-      <c r="P16" s="53"/>
-      <c r="Q16" s="53"/>
-      <c r="R16" s="53"/>
-      <c r="S16" s="53"/>
-      <c r="T16" s="53"/>
-      <c r="U16" s="53"/>
-      <c r="V16" s="53"/>
-      <c r="W16" s="53"/>
-      <c r="X16" s="53">
+      <c r="O16" s="40"/>
+      <c r="P16" s="40"/>
+      <c r="Q16" s="40"/>
+      <c r="R16" s="40"/>
+      <c r="S16" s="40"/>
+      <c r="T16" s="40"/>
+      <c r="U16" s="40"/>
+      <c r="V16" s="40"/>
+      <c r="W16" s="40"/>
+      <c r="X16" s="40">
         <v>25</v>
       </c>
-      <c r="Y16" s="53">
+      <c r="Y16" s="40">
         <v>35</v>
       </c>
-      <c r="Z16" s="53"/>
-      <c r="AA16" s="53"/>
-      <c r="AB16" s="53"/>
-      <c r="AC16" s="54">
+      <c r="Z16" s="40"/>
+      <c r="AA16" s="40"/>
+      <c r="AB16" s="40"/>
+      <c r="AC16" s="41">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="AD16" s="55">
+      <c r="AD16" s="42">
         <f>AC16*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1200</v>
       </c>
@@ -2579,27 +3775,27 @@
       <c r="N17" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="O17" s="53"/>
-      <c r="P17" s="53"/>
-      <c r="Q17" s="53"/>
-      <c r="R17" s="53"/>
-      <c r="S17" s="53"/>
-      <c r="T17" s="53"/>
-      <c r="U17" s="53"/>
-      <c r="V17" s="53"/>
-      <c r="W17" s="53"/>
-      <c r="X17" s="53"/>
-      <c r="Y17" s="53"/>
-      <c r="Z17" s="53">
+      <c r="O17" s="40"/>
+      <c r="P17" s="40"/>
+      <c r="Q17" s="40"/>
+      <c r="R17" s="40"/>
+      <c r="S17" s="40"/>
+      <c r="T17" s="40"/>
+      <c r="U17" s="40"/>
+      <c r="V17" s="40"/>
+      <c r="W17" s="40"/>
+      <c r="X17" s="40"/>
+      <c r="Y17" s="40"/>
+      <c r="Z17" s="40">
         <v>20</v>
       </c>
-      <c r="AA17" s="53"/>
-      <c r="AB17" s="53"/>
-      <c r="AC17" s="54">
+      <c r="AA17" s="40"/>
+      <c r="AB17" s="40"/>
+      <c r="AC17" s="41">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="AD17" s="55">
+      <c r="AD17" s="42">
         <f>AC17*'[1]Cost Estimate Summary'!$B$5</f>
         <v>400</v>
       </c>
@@ -2643,53 +3839,53 @@
       <c r="N18" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="O18" s="53">
+      <c r="O18" s="40">
         <v>5</v>
       </c>
-      <c r="P18" s="53">
+      <c r="P18" s="40">
         <v>5</v>
       </c>
-      <c r="Q18" s="53">
+      <c r="Q18" s="40">
         <v>5</v>
       </c>
-      <c r="R18" s="53">
+      <c r="R18" s="40">
         <v>5</v>
       </c>
-      <c r="S18" s="53">
+      <c r="S18" s="40">
         <v>5</v>
       </c>
-      <c r="T18" s="53">
+      <c r="T18" s="40">
         <v>5</v>
       </c>
-      <c r="U18" s="53">
+      <c r="U18" s="40">
         <v>5</v>
       </c>
-      <c r="V18" s="53">
+      <c r="V18" s="40">
         <v>5</v>
       </c>
-      <c r="W18" s="53">
+      <c r="W18" s="40">
         <v>5</v>
       </c>
-      <c r="X18" s="53">
+      <c r="X18" s="40">
         <v>5</v>
       </c>
-      <c r="Y18" s="53">
+      <c r="Y18" s="40">
         <v>5</v>
       </c>
-      <c r="Z18" s="53">
+      <c r="Z18" s="40">
         <v>5</v>
       </c>
-      <c r="AA18" s="53">
+      <c r="AA18" s="40">
         <v>5</v>
       </c>
-      <c r="AB18" s="53">
+      <c r="AB18" s="40">
         <v>5</v>
       </c>
-      <c r="AC18" s="54">
+      <c r="AC18" s="41">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="AD18" s="55">
+      <c r="AD18" s="42">
         <f>AC18*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1400</v>
       </c>
@@ -2733,29 +3929,29 @@
       <c r="N19" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="O19" s="53"/>
-      <c r="P19" s="53"/>
-      <c r="Q19" s="53"/>
-      <c r="R19" s="53"/>
-      <c r="S19" s="53"/>
-      <c r="T19" s="53"/>
-      <c r="U19" s="53"/>
-      <c r="V19" s="53"/>
-      <c r="W19" s="53"/>
-      <c r="X19" s="53"/>
-      <c r="Y19" s="53"/>
-      <c r="Z19" s="53"/>
-      <c r="AA19" s="53">
+      <c r="O19" s="40"/>
+      <c r="P19" s="40"/>
+      <c r="Q19" s="40"/>
+      <c r="R19" s="40"/>
+      <c r="S19" s="40"/>
+      <c r="T19" s="40"/>
+      <c r="U19" s="40"/>
+      <c r="V19" s="40"/>
+      <c r="W19" s="40"/>
+      <c r="X19" s="40"/>
+      <c r="Y19" s="40"/>
+      <c r="Z19" s="40"/>
+      <c r="AA19" s="40">
         <v>20</v>
       </c>
-      <c r="AB19" s="53">
+      <c r="AB19" s="40">
         <v>20</v>
       </c>
-      <c r="AC19" s="54">
+      <c r="AC19" s="41">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="AD19" s="55">
+      <c r="AD19" s="42">
         <f>AC19*'[1]Cost Estimate Summary'!$B$5</f>
         <v>800</v>
       </c>
@@ -2796,70 +3992,70 @@
         <f t="shared" si="5"/>
         <v>1400</v>
       </c>
-      <c r="N20" s="73" t="s">
+      <c r="N20" s="58" t="s">
         <v>97</v>
       </c>
-      <c r="O20" s="74">
+      <c r="O20" s="59">
         <f t="shared" ref="O20:AD20" si="6">SUM(O8:O19)</f>
         <v>30</v>
       </c>
-      <c r="P20" s="74">
+      <c r="P20" s="59">
         <f t="shared" si="6"/>
         <v>35</v>
       </c>
-      <c r="Q20" s="74">
+      <c r="Q20" s="59">
         <f t="shared" si="6"/>
         <v>50</v>
       </c>
-      <c r="R20" s="74">
+      <c r="R20" s="59">
         <f t="shared" si="6"/>
         <v>45</v>
       </c>
-      <c r="S20" s="74">
+      <c r="S20" s="59">
         <f t="shared" si="6"/>
         <v>55</v>
       </c>
-      <c r="T20" s="74">
+      <c r="T20" s="59">
         <f t="shared" si="6"/>
         <v>75</v>
       </c>
-      <c r="U20" s="74">
+      <c r="U20" s="59">
         <f t="shared" si="6"/>
         <v>85</v>
       </c>
-      <c r="V20" s="74">
+      <c r="V20" s="59">
         <f t="shared" si="6"/>
         <v>90</v>
       </c>
-      <c r="W20" s="74">
+      <c r="W20" s="59">
         <f t="shared" si="6"/>
         <v>105</v>
       </c>
-      <c r="X20" s="74">
+      <c r="X20" s="59">
         <f t="shared" si="6"/>
         <v>55</v>
       </c>
-      <c r="Y20" s="74">
+      <c r="Y20" s="59">
         <f t="shared" si="6"/>
         <v>40</v>
       </c>
-      <c r="Z20" s="74">
+      <c r="Z20" s="59">
         <f t="shared" si="6"/>
         <v>25</v>
       </c>
-      <c r="AA20" s="74">
+      <c r="AA20" s="59">
         <f t="shared" si="6"/>
         <v>25</v>
       </c>
-      <c r="AB20" s="74">
+      <c r="AB20" s="59">
         <f t="shared" si="6"/>
         <v>25</v>
       </c>
-      <c r="AC20" s="73">
+      <c r="AC20" s="58">
         <f t="shared" si="6"/>
         <v>740</v>
       </c>
-      <c r="AD20" s="75">
+      <c r="AD20" s="60">
         <f t="shared" si="6"/>
         <v>14800</v>
       </c>
@@ -2900,62 +4096,62 @@
         <f t="shared" si="5"/>
         <v>1000</v>
       </c>
-      <c r="N21" s="54" t="s">
+      <c r="N21" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="O21" s="56">
+      <c r="O21" s="43">
         <f>O20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>600</v>
       </c>
-      <c r="P21" s="56">
+      <c r="P21" s="43">
         <f>P20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>700</v>
       </c>
-      <c r="Q21" s="56">
+      <c r="Q21" s="43">
         <f>Q20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1000</v>
       </c>
-      <c r="R21" s="56">
+      <c r="R21" s="43">
         <f>R20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>900</v>
       </c>
-      <c r="S21" s="56">
+      <c r="S21" s="43">
         <f>S20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1100</v>
       </c>
-      <c r="T21" s="56">
+      <c r="T21" s="43">
         <f>T20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1500</v>
       </c>
-      <c r="U21" s="56">
+      <c r="U21" s="43">
         <f>U20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1700</v>
       </c>
-      <c r="V21" s="56">
+      <c r="V21" s="43">
         <f>V20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1800</v>
       </c>
-      <c r="W21" s="56">
+      <c r="W21" s="43">
         <f>W20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>2100</v>
       </c>
-      <c r="X21" s="56">
+      <c r="X21" s="43">
         <f>X20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>1100</v>
       </c>
-      <c r="Y21" s="56">
+      <c r="Y21" s="43">
         <f>Y20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>800</v>
       </c>
-      <c r="Z21" s="56">
+      <c r="Z21" s="43">
         <f>Z20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>500</v>
       </c>
-      <c r="AA21" s="56">
+      <c r="AA21" s="43">
         <f>AA20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>500</v>
       </c>
-      <c r="AB21" s="56">
+      <c r="AB21" s="43">
         <f>AB20*'[1]Cost Estimate Summary'!$B$5</f>
         <v>500</v>
       </c>
@@ -2963,36 +4159,36 @@
       <c r="AD21" s="17"/>
     </row>
     <row r="22" spans="1:30">
-      <c r="A22" s="69" t="s">
+      <c r="A22" s="54" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="70">
+      <c r="B22" s="55">
         <f>SUM(B9:B21)</f>
         <v>740</v>
       </c>
-      <c r="C22" s="71"/>
-      <c r="D22" s="72">
+      <c r="C22" s="56"/>
+      <c r="D22" s="57">
         <f>SUM(D9:D21)</f>
         <v>14800</v>
       </c>
-      <c r="E22" s="70">
+      <c r="E22" s="55">
         <f>SUM(E9:E21)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="71"/>
-      <c r="G22" s="72">
+      <c r="F22" s="56"/>
+      <c r="G22" s="57">
         <f>SUM(G9:G21)</f>
         <v>0</v>
       </c>
-      <c r="H22" s="72">
+      <c r="H22" s="57">
         <f>SUM(H9:H21)</f>
         <v>14800</v>
       </c>
-      <c r="I22" s="72">
+      <c r="I22" s="57">
         <f>SUM(I9:I21)</f>
         <v>2000</v>
       </c>
-      <c r="J22" s="72">
+      <c r="J22" s="57">
         <f>SUM(J9:J21)</f>
         <v>16800</v>
       </c>
@@ -3015,36 +4211,36 @@
       </c>
     </row>
     <row r="24" spans="1:30" ht="15.6">
-      <c r="A24" s="65" t="s">
+      <c r="A24" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="66">
+      <c r="B24" s="51">
         <f>B22</f>
         <v>740</v>
       </c>
-      <c r="C24" s="67"/>
-      <c r="D24" s="68">
+      <c r="C24" s="52"/>
+      <c r="D24" s="53">
         <f>D22</f>
         <v>14800</v>
       </c>
-      <c r="E24" s="66">
+      <c r="E24" s="51">
         <f>E22</f>
         <v>0</v>
       </c>
-      <c r="F24" s="67"/>
-      <c r="G24" s="68">
+      <c r="F24" s="52"/>
+      <c r="G24" s="53">
         <f>G22</f>
         <v>0</v>
       </c>
-      <c r="H24" s="68">
+      <c r="H24" s="53">
         <f>H22</f>
         <v>14800</v>
       </c>
-      <c r="I24" s="68">
+      <c r="I24" s="53">
         <f>I22</f>
         <v>2000</v>
       </c>
-      <c r="J24" s="68">
+      <c r="J24" s="53">
         <f>J22+J23</f>
         <v>18480</v>
       </c>
@@ -3073,91 +4269,92 @@
       <c r="J26" s="36"/>
     </row>
     <row r="27" spans="1:30">
-      <c r="A27" s="42" t="s">
+      <c r="A27" s="65" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="42"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="42"/>
-      <c r="F27" s="42"/>
-      <c r="G27" s="42"/>
-      <c r="H27" s="42"/>
-      <c r="I27" s="42"/>
-      <c r="J27" s="42"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="65"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="65"/>
+      <c r="F27" s="65"/>
+      <c r="G27" s="65"/>
+      <c r="H27" s="65"/>
+      <c r="I27" s="65"/>
+      <c r="J27" s="65"/>
     </row>
     <row r="28" spans="1:30">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="42"/>
+      <c r="B28" s="65"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="65"/>
+      <c r="H28" s="65"/>
+      <c r="I28" s="65"/>
+      <c r="J28" s="65"/>
     </row>
     <row r="29" spans="1:30">
-      <c r="A29" s="42" t="s">
+      <c r="A29" s="65" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="42"/>
-      <c r="I29" s="42"/>
-      <c r="J29" s="42"/>
+      <c r="B29" s="65"/>
+      <c r="C29" s="65"/>
+      <c r="D29" s="65"/>
+      <c r="E29" s="65"/>
+      <c r="F29" s="65"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="65"/>
+      <c r="I29" s="65"/>
+      <c r="J29" s="65"/>
     </row>
     <row r="30" spans="1:30">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="42"/>
+      <c r="B30" s="65"/>
+      <c r="C30" s="65"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="65"/>
+      <c r="F30" s="65"/>
+      <c r="G30" s="65"/>
+      <c r="H30" s="65"/>
+      <c r="I30" s="65"/>
+      <c r="J30" s="65"/>
     </row>
     <row r="31" spans="1:30">
-      <c r="A31" s="42" t="s">
+      <c r="A31" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="42"/>
-      <c r="C31" s="42"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="42"/>
-      <c r="J31" s="42"/>
+      <c r="B31" s="65"/>
+      <c r="C31" s="65"/>
+      <c r="D31" s="65"/>
+      <c r="E31" s="65"/>
+      <c r="F31" s="65"/>
+      <c r="G31" s="65"/>
+      <c r="H31" s="65"/>
+      <c r="I31" s="65"/>
+      <c r="J31" s="65"/>
     </row>
     <row r="32" spans="1:30">
-      <c r="A32" s="42" t="s">
+      <c r="A32" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="42"/>
+      <c r="B32" s="65"/>
+      <c r="C32" s="65"/>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="65"/>
+      <c r="G32" s="65"/>
+      <c r="H32" s="65"/>
+      <c r="I32" s="65"/>
+      <c r="J32" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A31:J31"/>
     <mergeCell ref="N5:AD5"/>
     <mergeCell ref="A32:J32"/>
     <mergeCell ref="A1:J1"/>
@@ -3174,8 +4371,146 @@
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A31:J31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11DC304E-A24C-4A26-826C-BBF7BE271E95}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="24.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" customWidth="1"/>
+    <col min="5" max="5" width="15.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="23.4">
+      <c r="A1" s="80" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="26">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" t="s">
+        <v>104</v>
+      </c>
+      <c r="E6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7" s="79">
+        <v>18480</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" s="79">
+        <v>18480</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="79">
+        <v>7407</v>
+      </c>
+      <c r="C8" s="79">
+        <v>32407</v>
+      </c>
+      <c r="D8" s="79">
+        <v>25887</v>
+      </c>
+      <c r="E8" s="79">
+        <v>32407</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" s="79">
+        <v>7545</v>
+      </c>
+      <c r="C9" s="79">
+        <v>48011</v>
+      </c>
+      <c r="D9" s="79">
+        <v>33432</v>
+      </c>
+      <c r="E9" s="79">
+        <v>80418</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" s="79">
+        <v>7684</v>
+      </c>
+      <c r="C10" s="79">
+        <v>66682</v>
+      </c>
+      <c r="D10" s="79">
+        <v>41116</v>
+      </c>
+      <c r="E10" s="79">
+        <v>147100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>